<commit_message>
added more test cases in login
</commit_message>
<xml_diff>
--- a/OkayGo/createWorker/non-lmd_onboarding_template (4).xlsx
+++ b/OkayGo/createWorker/non-lmd_onboarding_template (4).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/himanshu.tiwari/Okaygo/OkayGo/createWorker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8041F7F-A52E-E645-813F-2E17A3651FEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C27A1C8-4170-8F49-A205-6EBC14EA55FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="23260" windowHeight="12460" xr2:uid="{92AF1807-B58B-4D08-9DDB-0394152F5459}"/>
   </bookViews>
@@ -119,17 +119,17 @@
     <t>UAT Betterplace field verification</t>
   </si>
   <si>
-    <t>Automate</t>
-  </si>
-  <si>
-    <t>test</t>
+    <t>fg</t>
+  </si>
+  <si>
+    <t>yu</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -157,6 +157,12 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -201,13 +207,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -557,18 +564,18 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="23" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="4">
-        <v>9857654545</v>
+      <c r="C2" s="6">
+        <v>8478654907</v>
       </c>
       <c r="D2" s="5">
-        <v>958786454549</v>
+        <v>874674674884</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>7</v>

</xml_diff>